<commit_message>
feat(extras): update extra amenities photos and dimensions from catalog, add receptionist and mannequin photo
</commit_message>
<xml_diff>
--- a/STE-EXTRAS_RATE.xlsx
+++ b/STE-EXTRAS_RATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rebel\OneDrive\Documents\Projects\STE-feature-clean-code-assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F114F1C-6943-462A-9B75-DEF028E1485B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE0CCF5-7A00-408D-8A00-374907F8360A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{66487404-9CF7-4042-ADC4-BF91E97642DE}"/>
+    <workbookView xWindow="4800" yWindow="1350" windowWidth="14400" windowHeight="8722" xr2:uid="{66487404-9CF7-4042-ADC4-BF91E97642DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="56">
   <si>
     <t>INR Rates Listed</t>
   </si>
@@ -73,39 +73,15 @@
     <t>Rate Basis</t>
   </si>
   <si>
-    <t>Desk Table</t>
-  </si>
-  <si>
-    <t>1m x .5m x .75m</t>
-  </si>
-  <si>
     <t>Per day</t>
   </si>
   <si>
     <t>Glass Round Table</t>
   </si>
   <si>
-    <t>1m dia x .75m</t>
-  </si>
-  <si>
-    <t>White Chair</t>
-  </si>
-  <si>
-    <t>Cushioned Chair</t>
-  </si>
-  <si>
     <t>Sofa Single Seat</t>
   </si>
   <si>
-    <t>Sofa Double Seat</t>
-  </si>
-  <si>
-    <t>Sofa Three Seat</t>
-  </si>
-  <si>
-    <t>Brochure Rack</t>
-  </si>
-  <si>
     <t>Pedestrian Fan</t>
   </si>
   <si>
@@ -127,10 +103,118 @@
     <t>Metal Halide</t>
   </si>
   <si>
-    <t xml:space="preserve">Plasma with Stand 32 INCH </t>
-  </si>
-  <si>
-    <t>Garment Stand</t>
+    <t>System Table (Desk Table)</t>
+  </si>
+  <si>
+    <t>1m*0.5m*0.75m ht</t>
+  </si>
+  <si>
+    <t>Wooden Table with cover</t>
+  </si>
+  <si>
+    <t>5'x2.5'</t>
+  </si>
+  <si>
+    <t>2'8" Ø &amp; 2'6"ht</t>
+  </si>
+  <si>
+    <t>Exhibition Chairs (White Chair)</t>
+  </si>
+  <si>
+    <t>Standard exhibition seating</t>
+  </si>
+  <si>
+    <t>Stake Chair (Cushioned Chair)</t>
+  </si>
+  <si>
+    <t>Cushioned conference chair</t>
+  </si>
+  <si>
+    <t>Apple chair</t>
+  </si>
+  <si>
+    <t>Modern designer seating</t>
+  </si>
+  <si>
+    <t>Plush armchair</t>
+  </si>
+  <si>
+    <t>2 Seater Sofa (Sofa Double Seat)</t>
+  </si>
+  <si>
+    <t>2-seater luxury lounge sofa</t>
+  </si>
+  <si>
+    <t>3 Seater Sofa (Sofa Three Seat)</t>
+  </si>
+  <si>
+    <t>3-seater spacious lounge sofa</t>
+  </si>
+  <si>
+    <t>Rectangle Tipoi (Glass Centre Table)</t>
+  </si>
+  <si>
+    <t>Glass top lounge center table</t>
+  </si>
+  <si>
+    <t>Display Glass Counter Show case (without lock) No light</t>
+  </si>
+  <si>
+    <t>37.50"*18"*39"h</t>
+  </si>
+  <si>
+    <t>Display Glass Counter show case (with lock) No light</t>
+  </si>
+  <si>
+    <t>Tall showcase (without lock) No light</t>
+  </si>
+  <si>
+    <t>37.50"*18"*84"h</t>
+  </si>
+  <si>
+    <t>Tall showcase (with lock) No light</t>
+  </si>
+  <si>
+    <t>Brochure stand (Brochure Rack)</t>
+  </si>
+  <si>
+    <t>Folding catalogue display stand</t>
+  </si>
+  <si>
+    <t>High power pedestal fan</t>
+  </si>
+  <si>
+    <t>1m*10"</t>
+  </si>
+  <si>
+    <t>Spotlight / 50W LED fixture</t>
+  </si>
+  <si>
+    <t>Plasma with Stand 32 INCH</t>
+  </si>
+  <si>
+    <t>32-inch display with floor stand</t>
+  </si>
+  <si>
+    <t>Garment stand (Single rod)</t>
+  </si>
+  <si>
+    <t>4.5'w*5.5'ht</t>
+  </si>
+  <si>
+    <t>Garment stand (Double rod)</t>
+  </si>
+  <si>
+    <t>Receptionist</t>
+  </si>
+  <si>
+    <t>Professional stall receptionist / hostess (per day)</t>
+  </si>
+  <si>
+    <t>Mannequin</t>
+  </si>
+  <si>
+    <t>Full-body garment display mannequin</t>
   </si>
 </sst>
 </file>
@@ -213,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -225,15 +309,27 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -255,37 +351,48 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>297180</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>982980</xdr:rowOff>
+      <xdr:colOff>307181</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1307306</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="cc0f2cc1-6e27-43c8-bef2-6ba84888391a">
+        <xdr:cNvPr id="4" name="Pic_DP 01">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EA7C833-A314-46D2-903F-07D879CB3C84}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{828B22DF-3653-B5CF-479A-A82516BBCB39}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4702493" y="887730"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="307181" y="636588"/>
+          <a:ext cx="1000125" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -293,38 +400,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>297180</xdr:colOff>
+      <xdr:colOff>311386</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1303102</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="50d9baad-b5c3-4388-8336-ba3cd927295e">
+        <xdr:cNvPr id="8" name="Pic_DP 02">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1681E43-4BCE-4CDB-B5FB-79370922DF78}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17B74224-9B6B-0455-9DB6-E4A67D21DE36}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4702493" y="1654493"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="311386" y="1460500"/>
+          <a:ext cx="991716" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -332,38 +450,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>129540</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>754380</xdr:rowOff>
+      <xdr:colOff>406633</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1207854</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="3ab8a5b6-b4ac-49ef-bebc-3e615312be6f">
+        <xdr:cNvPr id="12" name="Pic_DP 03">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E6A7AA4-BC6C-4CC0-BFEF-A021EF3E68BB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0920FF1-0A65-BE06-0CC7-0235C80E6B95}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4534853" y="2378393"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="406633" y="2284413"/>
+          <a:ext cx="801221" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -371,38 +500,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:colOff>432851</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1181636</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="d8c09a8f-bc89-44b3-a01c-5c3b5dd9f10d">
+        <xdr:cNvPr id="16" name="Pic_DP 04">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AE74FD0-4E17-4412-85C6-2A9762729C48}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5D22B72-97FD-4C28-9591-6C2CFB30CB64}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4557713" y="3162300"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="432851" y="3108325"/>
+          <a:ext cx="748785" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -410,38 +550,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>167640</xdr:colOff>
+      <xdr:colOff>393143</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>236220</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1221344</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="7d72b60b-b8d1-4403-ba90-f7a88661b703">
+        <xdr:cNvPr id="19" name="Pic_DP 05">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B277BE85-CE53-48C8-B6D9-C9B0C1D038C7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B2AE0CC-F030-4C7D-F9CC-840D88EA6E2C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4572953" y="4103370"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="393143" y="3932238"/>
+          <a:ext cx="828201" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -449,38 +600,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>259080</xdr:colOff>
+      <xdr:colOff>510580</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1103908</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="2143ea4a-d3ab-4c06-a876-e78cbcb3a62e">
+        <xdr:cNvPr id="22" name="Pic_DP 06">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95E3EF20-3451-4977-B84D-E48DFD375F41}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{233917B7-546E-3CD3-B645-44A674C0CF93}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4664393" y="4903470"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="510580" y="4756150"/>
+          <a:ext cx="593328" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -488,38 +650,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>274320</xdr:colOff>
+      <xdr:colOff>325702</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="e9bab8cd-cd6f-4924-9fcc-398bc3ede123">
+        <xdr:cNvPr id="25" name="Pic_DP 08">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{299CAB8D-996B-4B87-A021-BD284006AD39}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{986EF37E-3A49-3A38-39CB-B1161D0D5648}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4679633" y="5830253"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="325702" y="5580063"/>
+          <a:ext cx="963083" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -527,38 +700,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>274320</xdr:colOff>
+      <xdr:colOff>240029</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>175260</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1374458</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="fb5b121a-f6ed-41bc-aaa2-32184b1b4c62">
+        <xdr:cNvPr id="27" name="Pic_DP 09">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8DF7810-5607-441E-AA85-E452094A9C32}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11C9C8C3-23A0-4258-366F-766F68BBCB4D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4679633" y="6980873"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="240029" y="6403975"/>
+          <a:ext cx="1134429" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -566,38 +750,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>243840</xdr:colOff>
+      <xdr:colOff>246989</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>236220</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1367499</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="fa1829dd-e353-4446-8403-2dd84bf3cea0">
+        <xdr:cNvPr id="30" name="Pic_DP 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{661547D6-7B1B-4001-A63B-F079E091F1D3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{516B11EE-1A70-FB44-3300-7D38743225D0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4649153" y="8251508"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="246989" y="7227888"/>
+          <a:ext cx="1120510" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -605,38 +800,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>327660</xdr:colOff>
+      <xdr:colOff>139827</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>350520</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1474661</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="67a9715a-0374-4cbf-915b-6a13c25d5e73">
+        <xdr:cNvPr id="33" name="Pic_DP 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{950F9C47-4B11-4FC8-BABF-AA457524A1A2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA1F9D8E-9097-5F9F-AA88-94A0EF7E0D3D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4732973" y="9623108"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="139827" y="8051800"/>
+          <a:ext cx="1334834" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -644,38 +850,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>331527</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1282960</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="4914dc83-f6df-42fa-ac62-09577c43981b">
+        <xdr:cNvPr id="35" name="Pic_DP 12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECBD2D22-3E86-4B02-8922-ED02E10AD9C8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3B06836-7A3C-338E-9DE6-73B12C46F8C1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4405313" y="10758488"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="331527" y="8875713"/>
+          <a:ext cx="951433" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -683,38 +900,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>379207</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1235281</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="0f7b9bb9-4fb7-46ea-9b91-66f3768a6355">
+        <xdr:cNvPr id="38" name="Pic_DP 13">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6AF59D5-9BF8-4D97-B8AE-CAEDD8339F34}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF95FCF9-75F7-788A-2C77-4EFE8AEF4A61}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4405313" y="11877675"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="379207" y="9699625"/>
+          <a:ext cx="856074" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -722,38 +950,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>320040</xdr:colOff>
+      <xdr:colOff>516418</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>266700</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1098070</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="270156c7-5720-4cfd-9fa2-da41ccc2ff72">
+        <xdr:cNvPr id="41" name="Pic_DP 14">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DC20CE2-377A-4EA2-9118-3014E43A4F45}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19D6CE91-2A69-AC11-9FE5-AF46A67C05DD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4725353" y="13154025"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="516418" y="10523538"/>
+          <a:ext cx="581652" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -761,38 +1000,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>167640</xdr:colOff>
+      <xdr:colOff>516418</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1098070</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="1c952b9e-bb9b-45b5-bb5f-395cfc45b2ae">
+        <xdr:cNvPr id="43" name="Pic_DP 14A">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50A587E5-8D8C-4290-89B5-FD297A335810}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C740E0F1-C4BA-1EC3-6F77-66AD271D91E5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4572953" y="14547533"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="516418" y="11347450"/>
+          <a:ext cx="581652" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -800,38 +1050,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>198120</xdr:colOff>
+      <xdr:colOff>655481</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>959006</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="ec17ea3e-6f31-410b-8d6a-b0cccfc627fe">
+        <xdr:cNvPr id="46" name="Pic_DP 15">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F07A359-CA48-4911-8AF3-5E69380FF623}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB04D2EC-C12F-E1B7-C683-A394D570286A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4603433" y="15664815"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="655481" y="12171363"/>
+          <a:ext cx="303525" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -839,38 +1100,49 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
+      <xdr:colOff>325702</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>251460</xdr:rowOff>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1143000" cy="857250"/>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="39cdcd46-40ea-4cd5-aa02-0ed909ab1455">
+        <xdr:cNvPr id="49" name="Pic_DP 20">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59491D96-DC05-4E7F-A211-7BBF06712545}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E37A7587-78FD-E6F4-FD9A-B484B21D5CAD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4748213" y="16844010"/>
-          <a:ext cx="1143000" cy="857250"/>
+          <a:off x="325702" y="12995275"/>
+          <a:ext cx="963083" cy="722313"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -878,7 +1150,457 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>356286</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1258201</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Pic_DP 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20E54D6B-D91A-FD6A-AB9D-AA909FE1AAC9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="356286" y="13819188"/>
+          <a:ext cx="901915" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>325702</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Pic_DP 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B53660E-5352-E2DE-E4C6-20888E3CB9C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="325702" y="14643100"/>
+          <a:ext cx="963083" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>325702</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="57" name="Pic_DP 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B225316A-F949-93F0-6015-50ABEA925ABF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="325702" y="15467013"/>
+          <a:ext cx="963083" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>325702</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="59" name="Pic_DP 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F962B0C-ECD7-DC21-A42F-D5629DBEB3E3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="325702" y="16290925"/>
+          <a:ext cx="963083" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>325702</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1288785</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="62" name="Pic_DP 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{874A595D-8BF3-C5D9-EA02-01009CAEE8F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="325702" y="17114838"/>
+          <a:ext cx="963083" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>453731</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1160756</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="65" name="Pic_DP 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D37DDC1-0BCF-9985-A729-ED575C4204BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="453731" y="17938750"/>
+          <a:ext cx="707025" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>453939</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1160549</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="69" name="Pic_DP 27A">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{845DD87D-EC9F-A6BE-6147-A775E0BB6508}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="453939" y="18762663"/>
+          <a:ext cx="706610" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>446088</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1168401</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="73" name="Pic_DP 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA6388BC-DD6C-9B88-0255-177E719DAC70}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="446088" y="19586575"/>
+          <a:ext cx="722313" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>566205</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1048282</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>773113</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="75" name="Pic_DP 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55A0E22B-3499-C2D4-0130-069684E9C246}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="566205" y="20410488"/>
+          <a:ext cx="482077" cy="722313"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1199,14 +1921,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{214ACAE6-32F7-457F-9E74-9B849C58F9DD}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="31.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.86328125" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="41.86328125" customWidth="1"/>
+    <col min="1" max="1" width="22.59765625" customWidth="1"/>
+    <col min="2" max="2" width="32.59765625" customWidth="1"/>
+    <col min="3" max="3" width="28.59765625" customWidth="1"/>
+    <col min="4" max="4" width="20.59765625" customWidth="1"/>
+    <col min="5" max="6" width="14.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1215,19 +1937,19 @@
         <v>0</v>
       </c>
       <c r="C1" s="1">
-        <f>COUNT(D3:D18)</f>
-        <v>16</v>
+        <f>COUNT(D3:D27)</f>
+        <v>25</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="1">
-        <f>COUNT(E3:E18)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="194.25">
+        <f>COUNT(E3:E27)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="32" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1247,268 +1969,454 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.5">
+    <row r="3" spans="1:6" ht="65" customHeight="1">
       <c r="A3" s="3"/>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="7">
+        <v>600</v>
+      </c>
+      <c r="E3" s="8">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="65" customHeight="1">
+      <c r="A4" s="3"/>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="7">
+        <v>400</v>
+      </c>
+      <c r="E4" s="8">
+        <v>5</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="65" customHeight="1">
+      <c r="A5" s="3"/>
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="5">
+      <c r="C5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="7">
+        <v>1400</v>
+      </c>
+      <c r="E5" s="8">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="65" customHeight="1">
+      <c r="A6" s="3"/>
+      <c r="B6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="7">
+        <v>700</v>
+      </c>
+      <c r="E6" s="8">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="65" customHeight="1">
+      <c r="A7" s="3"/>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="7">
+        <v>700</v>
+      </c>
+      <c r="E7" s="8">
+        <v>8</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="65" customHeight="1">
+      <c r="A8" s="3"/>
+      <c r="B8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="7">
+        <v>500</v>
+      </c>
+      <c r="E8" s="8">
+        <v>6</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="65" customHeight="1">
+      <c r="A9" s="3"/>
+      <c r="B9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3000</v>
+      </c>
+      <c r="E9" s="8">
+        <v>33</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="65" customHeight="1">
+      <c r="A10" s="3"/>
+      <c r="B10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="7">
+        <v>5000</v>
+      </c>
+      <c r="E10" s="8">
+        <v>55</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="65" customHeight="1">
+      <c r="A11" s="3"/>
+      <c r="B11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="7">
+        <v>6000</v>
+      </c>
+      <c r="E11" s="8">
+        <v>66</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="65" customHeight="1">
+      <c r="A12" s="3"/>
+      <c r="B12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="7">
+        <v>1200</v>
+      </c>
+      <c r="E12" s="8">
+        <v>13</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="65" customHeight="1">
+      <c r="A13" s="3"/>
+      <c r="B13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="7">
+        <v>2500</v>
+      </c>
+      <c r="E13" s="8">
+        <v>28</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="65" customHeight="1">
+      <c r="A14" s="3"/>
+      <c r="B14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="7">
+        <v>3000</v>
+      </c>
+      <c r="E14" s="8">
+        <v>33</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="65" customHeight="1">
+      <c r="A15" s="3"/>
+      <c r="B15" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="7">
+        <v>4000</v>
+      </c>
+      <c r="E15" s="8">
+        <v>44</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="65" customHeight="1">
+      <c r="A16" s="3"/>
+      <c r="B16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="7">
+        <v>5000</v>
+      </c>
+      <c r="E16" s="8">
+        <v>55</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="65" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="7">
+        <v>1500</v>
+      </c>
+      <c r="E17" s="8">
+        <v>16</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="65" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="7">
+        <v>1500</v>
+      </c>
+      <c r="E18" s="8">
+        <v>16</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="65" customHeight="1">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="11">
         <v>600</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E19" s="11">
+        <v>6</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="65" customHeight="1">
+      <c r="A20" s="9"/>
+      <c r="B20" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="11">
+        <v>500</v>
+      </c>
+      <c r="E20" s="11">
+        <v>5</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="65" customHeight="1">
+      <c r="A21" s="9"/>
+      <c r="B21" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="11">
+        <v>250</v>
+      </c>
+      <c r="E21" s="11">
+        <v>3</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="65" customHeight="1">
+      <c r="A22" s="9"/>
+      <c r="B22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="11">
+        <v>1500</v>
+      </c>
+      <c r="E22" s="11">
+        <v>13</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="65" customHeight="1">
+      <c r="A23" s="9"/>
+      <c r="B23" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="11">
+        <v>3500</v>
+      </c>
+      <c r="E23" s="11">
+        <v>27</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="65" customHeight="1">
+      <c r="A24" s="9"/>
+      <c r="B24" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="11">
+        <v>900</v>
+      </c>
+      <c r="E24" s="11">
         <v>7</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="42.75">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="F24" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="65" customHeight="1">
+      <c r="A25" s="9"/>
+      <c r="B25" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="11">
+        <v>900</v>
+      </c>
+      <c r="E25" s="11">
+        <v>7</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="65" customHeight="1">
+      <c r="A26" s="9"/>
+      <c r="B26" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="11">
+        <v>1500</v>
+      </c>
+      <c r="E26" s="11">
+        <v>16</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="65" customHeight="1">
+      <c r="A27" s="9"/>
+      <c r="B27" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="11">
+        <v>1000</v>
+      </c>
+      <c r="E27" s="11">
         <v>12</v>
       </c>
-      <c r="D4" s="5">
-        <v>1400</v>
-      </c>
-      <c r="E4" s="6">
-        <v>15</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.5">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5">
-        <v>700</v>
-      </c>
-      <c r="E5" s="6">
-        <v>8</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="28.5">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5">
-        <v>700</v>
-      </c>
-      <c r="E6" s="6">
-        <v>8</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="42.75">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5">
-        <v>3000</v>
-      </c>
-      <c r="E7" s="6">
-        <v>33</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="42.75">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5">
-        <v>5000</v>
-      </c>
-      <c r="E8" s="6">
-        <v>55</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="28.5">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5">
-        <v>6000</v>
-      </c>
-      <c r="E9" s="6">
-        <v>66</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5">
-        <v>1200</v>
-      </c>
-      <c r="E10" s="6">
-        <v>13</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="28.5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5">
-        <v>1500</v>
-      </c>
-      <c r="E11" s="6">
-        <v>16</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="28.5">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5">
-        <v>1500</v>
-      </c>
-      <c r="E12" s="6">
-        <v>16</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="28.5">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="5">
-        <v>600</v>
-      </c>
-      <c r="E13" s="6">
-        <v>6</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="28.5">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="5">
-        <v>500</v>
-      </c>
-      <c r="E14" s="6">
-        <v>5</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="42.75">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="5">
-        <v>250</v>
-      </c>
-      <c r="E15" s="6">
-        <v>3</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="28.5">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5">
-        <v>1500</v>
-      </c>
-      <c r="E16" s="6">
-        <v>13</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="42.75">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="5">
-        <v>3500</v>
-      </c>
-      <c r="E17" s="6">
-        <v>27</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="28.5">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5">
-        <v>900</v>
-      </c>
-      <c r="E18" s="6">
-        <v>7</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>10</v>
+      <c r="F27" s="11" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>